<commit_message>
Cambios CSS, html, visualización y funcionalidad en Filtros. Adverentcias y Errores muestras - fechas.
</commit_message>
<xml_diff>
--- a/bateria_tests/muestras/plantilla_muestras_advertencias.xlsx
+++ b/bateria_tests/muestras/plantilla_muestras_advertencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\OneDrive\Documentos\Practicas_UOC\datos_muestras\bateria_tests\muestras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B83966-864B-4927-8307-8FF0C130B086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15566C05-E9B1-413E-AC1B-7C7B867B3626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{16C911DF-861F-4518-B37A-B68EA5D4CCB1}"/>
+    <workbookView xWindow="38340" yWindow="2490" windowWidth="28005" windowHeight="11175" xr2:uid="{16C911DF-861F-4518-B37A-B68EA5D4CCB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>ID Individuo</t>
   </si>
@@ -108,37 +108,28 @@
     <t>Estudio</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>alpha</t>
-  </si>
-  <si>
-    <t>epsilon</t>
-  </si>
-  <si>
-    <t>z</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>y</t>
-  </si>
-  <si>
-    <t>w</t>
-  </si>
-  <si>
-    <t>v</t>
-  </si>
-  <si>
-    <t>u</t>
-  </si>
-  <si>
-    <t>t</t>
-  </si>
-  <si>
-    <t>s</t>
+    <t>zz</t>
+  </si>
+  <si>
+    <t>yy</t>
+  </si>
+  <si>
+    <t>xx</t>
+  </si>
+  <si>
+    <t>we</t>
+  </si>
+  <si>
+    <t>vv</t>
+  </si>
+  <si>
+    <t>uu</t>
+  </si>
+  <si>
+    <t>tt</t>
+  </si>
+  <si>
+    <t>ss</t>
   </si>
 </sst>
 </file>
@@ -594,235 +585,43 @@
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" t="s">
-        <v>24</v>
-      </c>
-      <c r="R2">
-        <v>1</v>
-      </c>
-      <c r="S2">
-        <v>1</v>
-      </c>
-      <c r="T2">
-        <v>1</v>
-      </c>
-      <c r="U2">
-        <v>1</v>
-      </c>
-      <c r="V2" t="s">
-        <v>26</v>
-      </c>
-      <c r="W2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
         <v>29</v>
       </c>
-      <c r="Q3" t="s">
-        <v>24</v>
-      </c>
-      <c r="R3">
-        <v>1</v>
-      </c>
-      <c r="S3">
-        <v>1</v>
-      </c>
-      <c r="T3">
-        <v>1</v>
-      </c>
-      <c r="U3">
-        <v>1</v>
-      </c>
-      <c r="V3" t="s">
-        <v>26</v>
-      </c>
-      <c r="W3">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>24</v>
-      </c>
-      <c r="R4">
-        <v>1</v>
-      </c>
-      <c r="S4">
-        <v>1</v>
-      </c>
-      <c r="T4">
-        <v>1</v>
-      </c>
-      <c r="U4">
-        <v>1</v>
-      </c>
-      <c r="V4" t="s">
-        <v>26</v>
-      </c>
-      <c r="W4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" t="s">
-        <v>24</v>
-      </c>
-      <c r="R5">
-        <v>1</v>
-      </c>
-      <c r="S5">
-        <v>1</v>
-      </c>
-      <c r="T5">
-        <v>1</v>
-      </c>
-      <c r="U5">
-        <v>1</v>
-      </c>
-      <c r="V5" t="s">
-        <v>26</v>
-      </c>
-      <c r="W5">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
         <v>31</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>24</v>
-      </c>
-      <c r="R6">
-        <v>1</v>
-      </c>
-      <c r="S6">
-        <v>1</v>
-      </c>
-      <c r="T6">
-        <v>1</v>
-      </c>
-      <c r="U6">
-        <v>1</v>
-      </c>
-      <c r="V6" t="s">
-        <v>26</v>
-      </c>
-      <c r="W6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>24</v>
-      </c>
-      <c r="R7">
-        <v>1</v>
-      </c>
-      <c r="S7">
-        <v>1</v>
-      </c>
-      <c r="T7">
-        <v>1</v>
-      </c>
-      <c r="U7">
-        <v>2</v>
-      </c>
-      <c r="V7" t="s">
-        <v>25</v>
-      </c>
-      <c r="W7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>24</v>
-      </c>
-      <c r="R8">
-        <v>1</v>
-      </c>
-      <c r="S8">
-        <v>1</v>
-      </c>
-      <c r="T8">
-        <v>1</v>
-      </c>
-      <c r="U8">
-        <v>2</v>
-      </c>
-      <c r="V8" t="s">
-        <v>25</v>
-      </c>
-      <c r="W8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>2</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R9">
-        <v>1</v>
-      </c>
-      <c r="S9">
-        <v>1</v>
-      </c>
-      <c r="T9">
-        <v>1</v>
-      </c>
-      <c r="U9">
-        <v>2</v>
-      </c>
-      <c r="V9" t="s">
-        <v>25</v>
-      </c>
-      <c r="W9">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>